<commit_message>
Atualiza o arquivo 3DSB_Acompanhamento_CampusApp.xlsx e remove arquivo temporário
</commit_message>
<xml_diff>
--- a/docs/3DSB_Acompanhamento_CampusApp.xlsx
+++ b/docs/3DSB_Acompanhamento_CampusApp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\.github\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3979694D-AB44-4DAE-86D6-A00F1D5FE839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92961326-908F-46C6-A189-E52B49CF15C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1257" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1285" uniqueCount="551">
   <si>
     <t>Desenvolvimento de Dispositivos Móveis · IFTM Campus Uberlândia · Prof. Edson Angoti Júnior</t>
   </si>
@@ -1821,7 +1821,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1900,6 +1900,18 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1928,7 +1940,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2022,6 +2034,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2710,14 +2728,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0FDFF74-CD3B-4BC2-985D-0CD9C1F9EF2A}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.33203125" customWidth="1"/>
+    <col min="1" max="1" width="31.109375" customWidth="1"/>
     <col min="2" max="7" width="31.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -2862,7 +2880,180 @@
       </c>
       <c r="G7" s="34"/>
     </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>546</v>
+      </c>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="35"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="B12" s="36"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="35"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>539</v>
+      </c>
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
+        <v>542</v>
+      </c>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="B16" s="36"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="36"/>
+      <c r="F16" s="35"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" s="5" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" s="9" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" s="9" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" s="9" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="9" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" s="9" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" s="5" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" s="5" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" s="9" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" s="9" t="s">
+        <v>531</v>
+      </c>
+    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A11:A38">
+    <sortCondition ref="A11:A38"/>
+  </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>

</xml_diff>